<commit_message>
Fix Issue with House Lore Events
</commit_message>
<xml_diff>
--- a/00_Checklist.xlsx
+++ b/00_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paradox Interactive\Hearts of Iron IV\mod\FAB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F19E6587-9FEB-41D6-8E4C-823036A228B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C68B46-8D14-49DE-9924-D3C8919BA8DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="95">
   <si>
     <t>ITEM</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>Make S3 and S4 events add tension</t>
+  </si>
+  <si>
+    <t>Coring States Decision</t>
   </si>
 </sst>
 </file>
@@ -895,7 +898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.140625" style="5" bestFit="1" customWidth="1"/>
@@ -1814,6 +1817,11 @@
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>